<commit_message>
Revisi: perbaiki AC-09 salah label, lengkapi AC minimal 3 per story Must
</commit_message>
<xml_diff>
--- a/04-acceptance-criteria.xlsx
+++ b/04-acceptance-criteria.xlsx
@@ -80,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -89,6 +89,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -456,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -550,7 +553,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>US-02</t>
+          <t>US-01</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -560,17 +563,17 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>mahasiswa memilih alat, tanggal pinjam, dan tanggal rencana kembali</t>
+          <t>NIM mahasiswa masih memiliki denda atau alat yang belum dikembalikan</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>mahasiswa menekan submit</t>
+          <t>mahasiswa mengajukan peminjaman baru</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>sistem menyimpan pengajuan berstatus "Menunggu Verifikasi"</t>
+          <t>sistem menolak pengajuan dan menampilkan alasan penolakan</t>
         </is>
       </c>
     </row>
@@ -587,7 +590,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>tanggal rencana kembali lebih awal dari tanggal pinjam</t>
+          <t>mahasiswa memilih alat, tanggal pinjam, dan tanggal rencana kembali</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -597,7 +600,7 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>sistem menolak dan menampilkan pesan tanggal tidak valid</t>
+          <t>sistem menyimpan pengajuan berstatus "Menunggu Verifikasi"</t>
         </is>
       </c>
     </row>
@@ -614,7 +617,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>alat yang dipilih sedang dipinjam pada rentang tanggal yang sama</t>
+          <t>tanggal rencana kembali lebih awal dari tanggal pinjam</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -624,14 +627,14 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>sistem menolak pengajuan dan menampilkan info alat tidak tersedia</t>
+          <t>sistem menolak dan menampilkan pesan tanggal tidak valid</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>US-06</t>
+          <t>US-02</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -641,17 +644,17 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>pengajuan telah disetujui dan mahasiswa datang mengambil alat</t>
+          <t>alat yang dipilih sedang dipinjam pada rentang tanggal yang sama</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>laboran menandai KTM/KTP sudah diterima sebagai jaminan</t>
+          <t>mahasiswa menekan submit</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>status peminjaman berubah menjadi "Aktif" dan alat ditandai sedang dipinjam</t>
+          <t>sistem menolak pengajuan dan menampilkan info alat tidak tersedia</t>
         </is>
       </c>
     </row>
@@ -668,24 +671,24 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>mahasiswa datang mengambil alat tanpa membawa KTM/KTP</t>
+          <t>pengajuan telah disetujui dan mahasiswa datang mengambil alat</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>laboran mencoba memproses serah terima</t>
+          <t>laboran menandai KTM/KTP sudah diterima sebagai jaminan</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>sistem tidak mengizinkan status berubah menjadi "Aktif" sebelum jaminan tercatat</t>
+          <t>status peminjaman berubah menjadi "Aktif" dan alat ditandai sedang dipinjam</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>US-08</t>
+          <t>US-06</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -695,44 +698,206 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>tanggal saat ini melewati tanggal rencana kembali dan alat belum dikembalikan</t>
+          <t>mahasiswa datang mengambil alat tanpa membawa KTM/KTP</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>sistem menjalankan pengecekan harian</t>
+          <t>laboran mencoba memproses serah terima</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>sistem menghitung denda = jumlah hari telat × tarif denda per hari dan menampilkannya di akun mahasiswa</t>
+          <t>sistem tidak mengizinkan status berubah menjadi "Aktif" sebelum jaminan tercatat</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>US-06</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>AC-09</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>KTM/KTP sudah ditahan sebagai jaminan dan alat dikembalikan tepat waktu dalam kondisi baik</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>laboran memproses pengembalian</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>laboran dapat menandai jaminan dikembalikan dan status peminjaman menjadi "Selesai"</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
           <t>US-08</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>AC-09</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>AC-10</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>tanggal saat ini melewati tanggal rencana kembali dan alat belum dikembalikan</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>sistem menjalankan pengecekan harian</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>sistem menghitung denda = jumlah hari telat x tarif denda per hari dan menampilkannya di akun mahasiswa</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>US-08</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>AC-11</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>denda belum dibayar melewati batas waktu tertentu</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>sistem menjalankan pengecekan harian</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>akun mahasiswa ditandai tertahan dan tidak bisa mengajukan peminjaman baru</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>US-08</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>AC-12</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>alat dikembalikan tepat waktu</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>sistem menghitung status peminjaman</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>sistem tidak membuat denda apa pun untuk peminjaman tersebut</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>US-05</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>AC-13</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>mahasiswa membuka halaman denda</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>mahasiswa memilih bayar via QRIS</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
         <is>
           <t>sistem menampilkan kode QRIS dan menandai status lunas setelah pembayaran terkonfirmasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>US-05</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>AC-14</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>kode QRIS belum dibayar dalam batas waktu tertentu</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>mahasiswa kembali membuka halaman denda</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>sistem menampilkan status "Menunggu Pembayaran" dan mengirim pengingat</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>US-05</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>AC-15</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>pembayaran QRIS gagal atau timeout</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>mahasiswa kembali membuka halaman denda</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>sistem menampilkan opsi untuk membuat ulang kode QRIS</t>
         </is>
       </c>
     </row>

</xml_diff>